<commit_message>
Update S35 adopted and decay data, revise statistics
Added notes on questionable gamma transitions and updated transition assignments in S35_34s_d_pg.ens. Revised S35_adopted.ens by removing or updating questionable levels and transitions, clarifying multipolarities, and correcting cross-references and comments. Updated Statistics.xlsx with new data.
</commit_message>
<xml_diff>
--- a/Statistics.xlsx
+++ b/Statistics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\X\ND\ENSDF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AB17203-C1CF-495A-80AB-13042451DCA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E19DEF8C-80FD-4157-BCCE-8E6A1C55CB7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{E3F13E08-64ED-4767-9D40-D1E60D65A10A}"/>
   </bookViews>
@@ -1097,7 +1097,7 @@
         <v>309</v>
       </c>
       <c r="N9" s="5">
-        <v>20250731</v>
+        <v>20250820</v>
       </c>
       <c r="O9" s="5">
         <v>14</v>

</xml_diff>

<commit_message>
Update Cl35 datasets and add new PDF files
Revised ENS files for Cl35_35ar_ec_decay_1.7755_s, Cl35_36ar_n_d, and Cl35_40ca_mu-_nuang with updated data, comments, and formatting. Added new PDF files for Cl35_34s_d_n and Cl35_40ca_mu-_nuang, and updated Cl35_35ar_ec_decay_1.7755_s.pdf. Also updated Statistics.xlsx with new data.
</commit_message>
<xml_diff>
--- a/Statistics.xlsx
+++ b/Statistics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\X\ND\ENSDF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E19DEF8C-80FD-4157-BCCE-8E6A1C55CB7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E139E35A-B084-4A4F-B100-C37ED59F33CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{E3F13E08-64ED-4767-9D40-D1E60D65A10A}"/>
   </bookViews>
@@ -28,6 +28,9 @@
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -1150,11 +1153,11 @@
         <v>10</v>
       </c>
       <c r="L10" s="4">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="M10" s="8">
         <f t="shared" si="4"/>
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="O10" s="4">
         <f t="shared" si="8"/>
@@ -1406,7 +1409,7 @@
     <row r="15" spans="1:16" x14ac:dyDescent="0.3">
       <c r="L15" s="4">
         <f>SUM(L3:L14)</f>
-        <v>1476</v>
+        <v>1477</v>
       </c>
       <c r="O15" s="4">
         <f>SUM(O3:O14)</f>

</xml_diff>

<commit_message>
Update Cl35_adopted.ens formatting and data
Corrected formatting and clarified references in Cl35_adopted.ens for consistency. Also updated Statistics.xlsx with new data.
</commit_message>
<xml_diff>
--- a/Statistics.xlsx
+++ b/Statistics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\X\ND\ENSDF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{529C02D8-6C13-498E-9602-18A1F54D1C95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA6B8BEA-8762-45E5-841F-830C4BBBD332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{E3F13E08-64ED-4767-9D40-D1E60D65A10A}"/>
   </bookViews>
@@ -586,7 +586,7 @@
     <col min="12" max="12" width="5" style="1" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="13.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="9" style="4" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="3" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="3.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="12.21875" style="1" customWidth="1"/>
     <col min="17" max="16384" width="8.88671875" style="1"/>
   </cols>
@@ -1160,12 +1160,11 @@
         <v>591</v>
       </c>
       <c r="O10" s="4">
-        <f t="shared" si="8"/>
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="P10" s="8">
         <f t="shared" si="6"/>
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.3">
@@ -1413,7 +1412,13 @@
       </c>
       <c r="O15" s="4">
         <f>SUM(O3:O14)</f>
-        <v>83</v>
+        <v>87</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="O16" s="1">
+        <f>O15+COUNTA(B3:B14)</f>
+        <v>99</v>
       </c>
     </row>
     <row r="18" spans="2:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Revise A=35 evaluation and Cl-35 level assignments
Updated A35_cover.ens with a more comprehensive abstract, revised methodology, and acknowledgments. Improved spin/parity assignments and references for several Cl-35 levels in Cl35_adopted.ens and Cl35_34s_p_g.ens, clarifying experimental origins and analysis details. These changes enhance clarity, accuracy, and traceability of nuclear data for A=35 nuclides.
</commit_message>
<xml_diff>
--- a/Statistics.xlsx
+++ b/Statistics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\X\ND\ENSDF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA6B8BEA-8762-45E5-841F-830C4BBBD332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A303B6D-4877-4BA4-A6EE-FDB6E9978DF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{E3F13E08-64ED-4767-9D40-D1E60D65A10A}"/>
   </bookViews>
@@ -862,7 +862,7 @@
         <v>20250528</v>
       </c>
       <c r="O5" s="5">
-        <f t="shared" ref="O5:O10" si="8">I5</f>
+        <f t="shared" ref="O5" si="8">I5</f>
         <v>3</v>
       </c>
       <c r="P5" s="9">
@@ -1417,8 +1417,8 @@
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.3">
       <c r="O16" s="1">
-        <f>O15+COUNTA(B3:B14)</f>
-        <v>99</v>
+        <f>O15+COUNTA(B3:B13)</f>
+        <v>98</v>
       </c>
     </row>
     <row r="18" spans="2:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Update A=35 evaluation files and add 2025 evaluator notes
Added 'A35 Evaluator thoughts 2025.txt' with updated summary of nuclide studies and recent experimental results. Revised A35_cover.ens to reflect new findings and reorganized summary. Made minor corrections and updates to adopted data and comments in Al35, Ar35, P35, and S35 evaluation files. Relocated raw data files for Al35 and K35. Updated Statistics.xlsx with new data.
</commit_message>
<xml_diff>
--- a/Statistics.xlsx
+++ b/Statistics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\X\ND\ENSDF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A303B6D-4877-4BA4-A6EE-FDB6E9978DF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63822F33-1BCC-4BE6-9ACF-E7F8C4166237}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{E3F13E08-64ED-4767-9D40-D1E60D65A10A}"/>
   </bookViews>
@@ -216,7 +216,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -239,13 +239,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -715,7 +709,7 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="H3" s="9">
+      <c r="H3" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -723,7 +717,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J3" s="9">
+      <c r="J3" s="8">
         <f>I3</f>
         <v>0</v>
       </c>
@@ -733,7 +727,7 @@
       <c r="L3" s="5">
         <v>8</v>
       </c>
-      <c r="M3" s="9">
+      <c r="M3" s="8">
         <f t="shared" ref="M3:M14" si="4">L3</f>
         <v>8</v>
       </c>
@@ -744,7 +738,7 @@
         <f>I3</f>
         <v>0</v>
       </c>
-      <c r="P3" s="9">
+      <c r="P3" s="8">
         <f>O3</f>
         <v>0</v>
       </c>
@@ -776,7 +770,7 @@
         <f t="shared" si="5"/>
         <v>93</v>
       </c>
-      <c r="H4" s="9">
+      <c r="H4" s="8">
         <f t="shared" si="0"/>
         <v>93</v>
       </c>
@@ -784,7 +778,7 @@
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="J4" s="9">
+      <c r="J4" s="8">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
@@ -794,7 +788,7 @@
       <c r="L4" s="5">
         <v>31</v>
       </c>
-      <c r="M4" s="9">
+      <c r="M4" s="8">
         <f t="shared" si="4"/>
         <v>31</v>
       </c>
@@ -804,7 +798,7 @@
       <c r="O4" s="5">
         <v>2</v>
       </c>
-      <c r="P4" s="9">
+      <c r="P4" s="8">
         <f t="shared" ref="P4:P14" si="6">O4</f>
         <v>2</v>
       </c>
@@ -836,7 +830,7 @@
         <f t="shared" si="7"/>
         <v>243</v>
       </c>
-      <c r="H5" s="9">
+      <c r="H5" s="8">
         <f t="shared" si="0"/>
         <v>243</v>
       </c>
@@ -844,7 +838,7 @@
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="J5" s="9">
+      <c r="J5" s="8">
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
@@ -854,7 +848,7 @@
       <c r="L5" s="5">
         <v>57</v>
       </c>
-      <c r="M5" s="9">
+      <c r="M5" s="8">
         <f t="shared" si="4"/>
         <v>57</v>
       </c>
@@ -865,7 +859,7 @@
         <f t="shared" ref="O5" si="8">I5</f>
         <v>3</v>
       </c>
-      <c r="P5" s="9">
+      <c r="P5" s="8">
         <f t="shared" si="6"/>
         <v>3</v>
       </c>
@@ -897,7 +891,7 @@
         <f t="shared" si="9"/>
         <v>258</v>
       </c>
-      <c r="H6" s="9">
+      <c r="H6" s="8">
         <f t="shared" si="0"/>
         <v>258</v>
       </c>
@@ -905,7 +899,7 @@
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="J6" s="9">
+      <c r="J6" s="8">
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
@@ -915,7 +909,7 @@
       <c r="L6" s="5">
         <v>48</v>
       </c>
-      <c r="M6" s="9">
+      <c r="M6" s="8">
         <f t="shared" si="4"/>
         <v>48</v>
       </c>
@@ -925,7 +919,7 @@
       <c r="O6" s="5">
         <v>5</v>
       </c>
-      <c r="P6" s="9">
+      <c r="P6" s="8">
         <f t="shared" si="6"/>
         <v>5</v>
       </c>
@@ -957,7 +951,7 @@
         <f t="shared" si="10"/>
         <v>386</v>
       </c>
-      <c r="H7" s="9">
+      <c r="H7" s="8">
         <f t="shared" si="0"/>
         <v>386</v>
       </c>
@@ -965,7 +959,7 @@
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="J7" s="9">
+      <c r="J7" s="8">
         <f t="shared" si="2"/>
         <v>4</v>
       </c>
@@ -975,7 +969,7 @@
       <c r="L7" s="5">
         <v>65</v>
       </c>
-      <c r="M7" s="9">
+      <c r="M7" s="8">
         <f t="shared" si="4"/>
         <v>65</v>
       </c>
@@ -985,7 +979,7 @@
       <c r="O7" s="5">
         <v>6</v>
       </c>
-      <c r="P7" s="9">
+      <c r="P7" s="8">
         <f t="shared" si="6"/>
         <v>6</v>
       </c>
@@ -1017,7 +1011,7 @@
         <f t="shared" si="11"/>
         <v>398</v>
       </c>
-      <c r="H8" s="9">
+      <c r="H8" s="8">
         <f t="shared" si="0"/>
         <v>398</v>
       </c>
@@ -1025,7 +1019,7 @@
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
-      <c r="J8" s="9">
+      <c r="J8" s="8">
         <f t="shared" si="2"/>
         <v>7</v>
       </c>
@@ -1035,7 +1029,7 @@
       <c r="L8" s="5">
         <v>72</v>
       </c>
-      <c r="M8" s="9">
+      <c r="M8" s="8">
         <f t="shared" si="4"/>
         <v>72</v>
       </c>
@@ -1045,7 +1039,7 @@
       <c r="O8" s="5">
         <v>12</v>
       </c>
-      <c r="P8" s="9">
+      <c r="P8" s="8">
         <f t="shared" si="6"/>
         <v>12</v>
       </c>
@@ -1077,7 +1071,7 @@
         <f t="shared" si="12"/>
         <v>1043</v>
       </c>
-      <c r="H9" s="9">
+      <c r="H9" s="8">
         <f t="shared" si="0"/>
         <v>1043</v>
       </c>
@@ -1085,7 +1079,7 @@
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="J9" s="9">
+      <c r="J9" s="8">
         <f t="shared" si="2"/>
         <v>10</v>
       </c>
@@ -1095,7 +1089,7 @@
       <c r="L9" s="5">
         <v>309</v>
       </c>
-      <c r="M9" s="9">
+      <c r="M9" s="8">
         <f t="shared" si="4"/>
         <v>309</v>
       </c>
@@ -1105,35 +1099,35 @@
       <c r="O9" s="5">
         <v>14</v>
       </c>
-      <c r="P9" s="9">
+      <c r="P9" s="8">
         <f t="shared" si="6"/>
         <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A10" s="10">
+      <c r="A10" s="2">
         <v>17</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="4">
+      <c r="C10" s="5">
         <f t="shared" ref="C10:G10" si="13">C28</f>
         <v>352</v>
       </c>
-      <c r="D10" s="4">
+      <c r="D10" s="5">
         <f t="shared" si="13"/>
         <v>1136</v>
       </c>
-      <c r="E10" s="4">
+      <c r="E10" s="5">
         <f t="shared" si="13"/>
         <v>1042</v>
       </c>
-      <c r="F10" s="4">
+      <c r="F10" s="5">
         <f t="shared" si="13"/>
         <v>2396</v>
       </c>
-      <c r="G10" s="4">
+      <c r="G10" s="5">
         <f t="shared" si="13"/>
         <v>6896</v>
       </c>
@@ -1141,7 +1135,7 @@
         <f t="shared" si="0"/>
         <v>6896</v>
       </c>
-      <c r="I10" s="4">
+      <c r="I10" s="5">
         <f t="shared" si="1"/>
         <v>24</v>
       </c>
@@ -1149,17 +1143,20 @@
         <f t="shared" si="2"/>
         <v>24</v>
       </c>
-      <c r="K10" s="4">
+      <c r="K10" s="5">
         <v>10</v>
       </c>
-      <c r="L10" s="4">
+      <c r="L10" s="5">
         <v>591</v>
       </c>
       <c r="M10" s="8">
         <f t="shared" si="4"/>
         <v>591</v>
       </c>
-      <c r="O10" s="4">
+      <c r="N10" s="5">
+        <v>20251024</v>
+      </c>
+      <c r="O10" s="5">
         <v>28</v>
       </c>
       <c r="P10" s="8">
@@ -1194,7 +1191,7 @@
         <f t="shared" si="14"/>
         <v>639</v>
       </c>
-      <c r="H11" s="9">
+      <c r="H11" s="8">
         <f t="shared" si="0"/>
         <v>639</v>
       </c>
@@ -1202,7 +1199,7 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="J11" s="9">
+      <c r="J11" s="8">
         <f t="shared" si="2"/>
         <v>9</v>
       </c>
@@ -1212,7 +1209,7 @@
       <c r="L11" s="5">
         <v>193</v>
       </c>
-      <c r="M11" s="9">
+      <c r="M11" s="8">
         <f t="shared" si="4"/>
         <v>193</v>
       </c>
@@ -1222,7 +1219,7 @@
       <c r="O11" s="5">
         <v>11</v>
       </c>
-      <c r="P11" s="9">
+      <c r="P11" s="8">
         <f t="shared" si="6"/>
         <v>11</v>
       </c>
@@ -1254,7 +1251,7 @@
         <f t="shared" si="15"/>
         <v>165</v>
       </c>
-      <c r="H12" s="9">
+      <c r="H12" s="8">
         <f t="shared" si="0"/>
         <v>165</v>
       </c>
@@ -1262,7 +1259,7 @@
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="J12" s="9">
+      <c r="J12" s="8">
         <f t="shared" si="2"/>
         <v>2</v>
       </c>
@@ -1272,7 +1269,7 @@
       <c r="L12" s="5">
         <v>61</v>
       </c>
-      <c r="M12" s="9">
+      <c r="M12" s="8">
         <f t="shared" si="4"/>
         <v>61</v>
       </c>
@@ -1282,7 +1279,7 @@
       <c r="O12" s="5">
         <v>3</v>
       </c>
-      <c r="P12" s="9">
+      <c r="P12" s="8">
         <f t="shared" si="6"/>
         <v>3</v>
       </c>
@@ -1314,7 +1311,7 @@
         <f t="shared" si="16"/>
         <v>37</v>
       </c>
-      <c r="H13" s="9">
+      <c r="H13" s="8">
         <f t="shared" si="0"/>
         <v>37</v>
       </c>
@@ -1322,7 +1319,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J13" s="9">
+      <c r="J13" s="8">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -1332,7 +1329,7 @@
       <c r="L13" s="5">
         <v>33</v>
       </c>
-      <c r="M13" s="9">
+      <c r="M13" s="8">
         <f t="shared" si="4"/>
         <v>33</v>
       </c>
@@ -1342,7 +1339,7 @@
       <c r="O13" s="5">
         <v>3</v>
       </c>
-      <c r="P13" s="9">
+      <c r="P13" s="8">
         <f t="shared" si="6"/>
         <v>3</v>
       </c>
@@ -1374,7 +1371,7 @@
         <f t="shared" si="16"/>
         <v>0</v>
       </c>
-      <c r="H14" s="9">
+      <c r="H14" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -1382,7 +1379,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J14" s="9">
+      <c r="J14" s="8">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -1392,7 +1389,7 @@
       <c r="L14" s="5">
         <v>9</v>
       </c>
-      <c r="M14" s="9">
+      <c r="M14" s="8">
         <f t="shared" si="4"/>
         <v>9</v>
       </c>
@@ -1400,7 +1397,7 @@
         <v>20250506</v>
       </c>
       <c r="O14" s="5"/>
-      <c r="P14" s="9">
+      <c r="P14" s="8">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Update Ca34 and K34 adopted data and add new PDFs
Revised adopted level and structure information for Ca34 and K34 in .ens files, including updated references and clarifications. Added new PDF files for K34 (adopted and 9be_37ca_x) and updated Ca34 adopted PDF. Also updated Statistics.xlsx with new data.
</commit_message>
<xml_diff>
--- a/Statistics.xlsx
+++ b/Statistics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\X\ND\ENSDF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4269248-585E-44D4-BE8B-4CA1DEC5506D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AFDFC73-A004-4B0B-8008-FBA0B0F6823D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{E3F13E08-64ED-4767-9D40-D1E60D65A10A}"/>
   </bookViews>
@@ -240,7 +240,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -252,6 +252,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -589,7 +592,7 @@
     <col min="9" max="10" width="12.77734375" style="1" customWidth="1"/>
     <col min="11" max="11" width="4.21875" style="1" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="12.77734375" style="1" customWidth="1"/>
-    <col min="13" max="13" width="8.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="3.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="12.21875" style="1" customWidth="1"/>
     <col min="16" max="16384" width="8.88671875" style="1"/>
@@ -1054,7 +1057,7 @@
         <v>67</v>
       </c>
       <c r="L17" s="3">
-        <f>K17</f>
+        <f t="shared" ref="L17:L27" si="3">K17</f>
         <v>67</v>
       </c>
       <c r="M17" s="4"/>
@@ -1075,7 +1078,7 @@
         <v>40</v>
       </c>
       <c r="L18" s="3">
-        <f>K18</f>
+        <f t="shared" si="3"/>
         <v>40</v>
       </c>
       <c r="M18" s="4"/>
@@ -1096,7 +1099,7 @@
         <v>196</v>
       </c>
       <c r="L19" s="3">
-        <f>K19</f>
+        <f t="shared" si="3"/>
         <v>196</v>
       </c>
       <c r="M19" s="4"/>
@@ -1117,7 +1120,7 @@
         <v>67</v>
       </c>
       <c r="L20" s="3">
-        <f>K20</f>
+        <f t="shared" si="3"/>
         <v>67</v>
       </c>
       <c r="M20" s="4"/>
@@ -1138,7 +1141,7 @@
         <v>245</v>
       </c>
       <c r="L21" s="3">
-        <f>K21</f>
+        <f t="shared" si="3"/>
         <v>245</v>
       </c>
       <c r="M21" s="4"/>
@@ -1159,7 +1162,7 @@
         <v>107</v>
       </c>
       <c r="L22" s="3">
-        <f>K22</f>
+        <f t="shared" si="3"/>
         <v>107</v>
       </c>
       <c r="M22" s="4"/>
@@ -1180,7 +1183,7 @@
         <v>539</v>
       </c>
       <c r="L23" s="3">
-        <f>K23</f>
+        <f t="shared" si="3"/>
         <v>539</v>
       </c>
       <c r="M23" s="4"/>
@@ -1201,7 +1204,7 @@
         <v>461</v>
       </c>
       <c r="L24" s="3">
-        <f>K24</f>
+        <f t="shared" si="3"/>
         <v>461</v>
       </c>
       <c r="M24" s="4"/>
@@ -1222,7 +1225,7 @@
         <v>209</v>
       </c>
       <c r="L25" s="3">
-        <f>K25</f>
+        <f t="shared" si="3"/>
         <v>209</v>
       </c>
       <c r="M25" s="4"/>
@@ -1231,26 +1234,34 @@
       <c r="B26" s="1" t="s">
         <v>25</v>
       </c>
+      <c r="H26" s="1">
+        <v>1</v>
+      </c>
       <c r="I26" s="3">
         <f>G26</f>
         <v>0</v>
       </c>
       <c r="J26" s="3">
         <f>H26</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K26" s="4">
         <v>24</v>
       </c>
       <c r="L26" s="3">
-        <f>K26</f>
+        <f t="shared" si="3"/>
         <v>24</v>
       </c>
-      <c r="M26" s="4"/>
+      <c r="M26" s="5">
+        <v>45972</v>
+      </c>
     </row>
     <row r="27" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B27" s="1" t="s">
         <v>33</v>
+      </c>
+      <c r="H27" s="1">
+        <v>0</v>
       </c>
       <c r="I27" s="4"/>
       <c r="J27" s="4"/>
@@ -1258,10 +1269,12 @@
         <v>82</v>
       </c>
       <c r="L27" s="3">
-        <f>K27</f>
+        <f t="shared" si="3"/>
         <v>82</v>
       </c>
-      <c r="M27" s="4"/>
+      <c r="M27" s="5">
+        <v>45971</v>
+      </c>
     </row>
     <row r="28" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B28" s="1" t="s">
@@ -1874,7 +1887,7 @@
         <v>8</v>
       </c>
       <c r="L16" s="3">
-        <f>K16</f>
+        <f t="shared" ref="L16:L26" si="2">K16</f>
         <v>8</v>
       </c>
       <c r="M16" s="4">
@@ -1904,18 +1917,18 @@
         <v>2</v>
       </c>
       <c r="I17" s="3">
-        <f t="shared" ref="I17:J25" si="2">G17</f>
+        <f t="shared" ref="I17:J25" si="3">G17</f>
         <v>117</v>
       </c>
       <c r="J17" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>2</v>
       </c>
       <c r="K17" s="4">
         <v>31</v>
       </c>
       <c r="L17" s="3">
-        <f>K17</f>
+        <f t="shared" si="2"/>
         <v>31</v>
       </c>
       <c r="M17" s="4">
@@ -1945,18 +1958,18 @@
         <v>3</v>
       </c>
       <c r="I18" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>328</v>
       </c>
       <c r="J18" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>3</v>
       </c>
       <c r="K18" s="4">
         <v>57</v>
       </c>
       <c r="L18" s="3">
-        <f>K18</f>
+        <f t="shared" si="2"/>
         <v>57</v>
       </c>
       <c r="M18" s="4">
@@ -1986,18 +1999,18 @@
         <v>5</v>
       </c>
       <c r="I19" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>379</v>
       </c>
       <c r="J19" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>5</v>
       </c>
       <c r="K19" s="4">
         <v>48</v>
       </c>
       <c r="L19" s="3">
-        <f>K19</f>
+        <f t="shared" si="2"/>
         <v>48</v>
       </c>
       <c r="M19" s="4">
@@ -2027,18 +2040,18 @@
         <v>6</v>
       </c>
       <c r="I20" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>565</v>
       </c>
       <c r="J20" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>6</v>
       </c>
       <c r="K20" s="4">
         <v>65</v>
       </c>
       <c r="L20" s="3">
-        <f>K20</f>
+        <f t="shared" si="2"/>
         <v>65</v>
       </c>
       <c r="M20" s="4">
@@ -2068,18 +2081,18 @@
         <v>12</v>
       </c>
       <c r="I21" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>934</v>
       </c>
       <c r="J21" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>12</v>
       </c>
       <c r="K21" s="4">
         <v>72</v>
       </c>
       <c r="L21" s="3">
-        <f>K21</f>
+        <f t="shared" si="2"/>
         <v>72</v>
       </c>
       <c r="M21" s="4">
@@ -2109,18 +2122,18 @@
         <v>14</v>
       </c>
       <c r="I22" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>2437</v>
       </c>
       <c r="J22" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>14</v>
       </c>
       <c r="K22" s="4">
         <v>309</v>
       </c>
       <c r="L22" s="3">
-        <f>K22</f>
+        <f t="shared" si="2"/>
         <v>309</v>
       </c>
       <c r="M22" s="4">
@@ -2150,18 +2163,18 @@
         <v>28</v>
       </c>
       <c r="I23" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>8616</v>
       </c>
       <c r="J23" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>28</v>
       </c>
       <c r="K23" s="4">
         <v>591</v>
       </c>
       <c r="L23" s="3">
-        <f>K23</f>
+        <f t="shared" si="2"/>
         <v>591</v>
       </c>
       <c r="M23" s="4">
@@ -2191,18 +2204,18 @@
         <v>11</v>
       </c>
       <c r="I24" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1232</v>
       </c>
       <c r="J24" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>11</v>
       </c>
       <c r="K24" s="4">
         <v>193</v>
       </c>
       <c r="L24" s="3">
-        <f>K24</f>
+        <f t="shared" si="2"/>
         <v>193</v>
       </c>
       <c r="M24" s="4">
@@ -2232,18 +2245,18 @@
         <v>3</v>
       </c>
       <c r="I25" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>307</v>
       </c>
       <c r="J25" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>3</v>
       </c>
       <c r="K25" s="4">
         <v>61</v>
       </c>
       <c r="L25" s="3">
-        <f>K25</f>
+        <f t="shared" si="2"/>
         <v>61</v>
       </c>
       <c r="M25" s="4">
@@ -2284,7 +2297,7 @@
         <v>33</v>
       </c>
       <c r="L26" s="3">
-        <f>K26</f>
+        <f t="shared" si="2"/>
         <v>33</v>
       </c>
       <c r="M26" s="4">
@@ -2596,7 +2609,7 @@
         <v>6</v>
       </c>
       <c r="I5" s="3">
-        <f t="shared" ref="I5:J13" si="0">G5</f>
+        <f t="shared" ref="I5:I13" si="0">G5</f>
         <v>257</v>
       </c>
       <c r="J5" s="3">

</xml_diff>

<commit_message>
Update ENSDF data and statistics for Ar34 reactions
Added new author and citation information to Ar34_32s_3he_n.ens and Ar34_3he_32s_ng_32s_3he_ng.ens, updated dataset identifiers and cut dates, and modified Statistics.xlsx to reflect the latest data.
</commit_message>
<xml_diff>
--- a/Statistics.xlsx
+++ b/Statistics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\X\ND\ENSDF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AFDFC73-A004-4B0B-8008-FBA0B0F6823D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F50A322-EA3B-4529-B430-7B69D4CF7CF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{E3F13E08-64ED-4767-9D40-D1E60D65A10A}"/>
   </bookViews>
@@ -1213,13 +1213,16 @@
       <c r="B25" s="1" t="s">
         <v>32</v>
       </c>
+      <c r="H25" s="1">
+        <v>9</v>
+      </c>
       <c r="I25" s="3">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="J25" s="3">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="K25" s="4">
         <v>209</v>

</xml_diff>

<commit_message>
Update Statistics.xlsx with revised data
</commit_message>
<xml_diff>
--- a/Statistics.xlsx
+++ b/Statistics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\X\ND\ENSDF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F50A322-EA3B-4529-B430-7B69D4CF7CF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8478164-EDB1-4C5A-B366-FA9DEFD3D23E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{E3F13E08-64ED-4767-9D40-D1E60D65A10A}"/>
   </bookViews>
@@ -1213,16 +1213,31 @@
       <c r="B25" s="1" t="s">
         <v>32</v>
       </c>
+      <c r="C25" s="1">
+        <v>42</v>
+      </c>
+      <c r="D25" s="1">
+        <v>26</v>
+      </c>
+      <c r="E25" s="1">
+        <v>132</v>
+      </c>
+      <c r="F25" s="1">
+        <v>67</v>
+      </c>
+      <c r="G25" s="1">
+        <v>840</v>
+      </c>
       <c r="H25" s="1">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I25" s="3">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>840</v>
       </c>
       <c r="J25" s="3">
         <f t="shared" si="2"/>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K25" s="4">
         <v>209</v>
@@ -1231,7 +1246,9 @@
         <f t="shared" si="3"/>
         <v>209</v>
       </c>
-      <c r="M25" s="4"/>
+      <c r="M25" s="5">
+        <v>45995</v>
+      </c>
     </row>
     <row r="26" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B26" s="1" t="s">

</xml_diff>

<commit_message>
Move and rename Cl34 data files, clean up old versions
Renamed Cl34 data files from .old and .xundl extensions to .ens in a new directory structure under A34/Cl34/new/. Archived the original files in A34/Cl34/old/. Also removed obsolete files AverageTool_22January2025.jar and test.txt, and updated Statistics.xlsx.
</commit_message>
<xml_diff>
--- a/Statistics.xlsx
+++ b/Statistics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\X\ND\ENSDF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8478164-EDB1-4C5A-B366-FA9DEFD3D23E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1816A8B7-6687-4639-98A5-F0402059BEFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{E3F13E08-64ED-4767-9D40-D1E60D65A10A}"/>
   </bookViews>
@@ -1192,13 +1192,16 @@
       <c r="B24" s="1" t="s">
         <v>31</v>
       </c>
+      <c r="H24" s="1">
+        <v>23</v>
+      </c>
       <c r="I24" s="3">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="J24" s="3">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="K24" s="4">
         <v>461</v>

</xml_diff>

<commit_message>
Remove Ar34_35ca_ecp_decay_25.7_ms.ens and update Cl34_35cl_d_t.ens
Deleted the Ar34_35ca_ecp_decay_25.7_ms.ens file and made a minor edit to the Cl34_35cl_d_t.ens file for clarity in the description of the 1981Bh04 experiment. Updated Statistics.xlsx with new data.
</commit_message>
<xml_diff>
--- a/Statistics.xlsx
+++ b/Statistics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\X\ND\ENSDF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1816A8B7-6687-4639-98A5-F0402059BEFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46AD183F-6BB6-41F0-8715-4A88C93BFA50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{E3F13E08-64ED-4767-9D40-D1E60D65A10A}"/>
   </bookViews>
@@ -1060,7 +1060,9 @@
         <f t="shared" ref="L17:L27" si="3">K17</f>
         <v>67</v>
       </c>
-      <c r="M17" s="4"/>
+      <c r="M17" s="5">
+        <v>46179</v>
+      </c>
     </row>
     <row r="18" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B18" s="1" t="s">
@@ -1081,7 +1083,9 @@
         <f t="shared" si="3"/>
         <v>40</v>
       </c>
-      <c r="M18" s="4"/>
+      <c r="M18" s="5">
+        <v>46156</v>
+      </c>
     </row>
     <row r="19" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B19" s="1" t="s">
@@ -1102,7 +1106,9 @@
         <f t="shared" si="3"/>
         <v>196</v>
       </c>
-      <c r="M19" s="4"/>
+      <c r="M19" s="5">
+        <v>46133</v>
+      </c>
     </row>
     <row r="20" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B20" s="1" t="s">
@@ -1123,7 +1129,9 @@
         <f t="shared" si="3"/>
         <v>67</v>
       </c>
-      <c r="M20" s="4"/>
+      <c r="M20" s="5">
+        <v>46110</v>
+      </c>
     </row>
     <row r="21" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B21" s="1" t="s">
@@ -1144,7 +1152,9 @@
         <f t="shared" si="3"/>
         <v>245</v>
       </c>
-      <c r="M21" s="4"/>
+      <c r="M21" s="5">
+        <v>46087</v>
+      </c>
     </row>
     <row r="22" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B22" s="1" t="s">
@@ -1165,7 +1175,9 @@
         <f t="shared" si="3"/>
         <v>107</v>
       </c>
-      <c r="M22" s="4"/>
+      <c r="M22" s="5">
+        <v>46064</v>
+      </c>
     </row>
     <row r="23" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B23" s="1" t="s">
@@ -1186,7 +1198,9 @@
         <f t="shared" si="3"/>
         <v>539</v>
       </c>
-      <c r="M23" s="4"/>
+      <c r="M23" s="5">
+        <v>46041</v>
+      </c>
     </row>
     <row r="24" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B24" s="1" t="s">
@@ -1210,7 +1224,9 @@
         <f t="shared" si="3"/>
         <v>461</v>
       </c>
-      <c r="M24" s="4"/>
+      <c r="M24" s="5">
+        <v>46018</v>
+      </c>
     </row>
     <row r="25" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B25" s="1" t="s">

</xml_diff>

<commit_message>
Update Cl34_33s_3he_d.ens text and Statistics.xlsx data
Improved clarity and consistency in Cl34_33s_3he_d.ens by rephrasing descriptions and consolidating related information onto single lines. Updated Statistics.xlsx with new or revised data.
</commit_message>
<xml_diff>
--- a/Statistics.xlsx
+++ b/Statistics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\X\ND\ENSDF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46AD183F-6BB6-41F0-8715-4A88C93BFA50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A781ADA-B8CF-4AF6-A8A3-CEB3DE3A9724}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{E3F13E08-64ED-4767-9D40-D1E60D65A10A}"/>
   </bookViews>
@@ -1248,7 +1248,7 @@
         <v>840</v>
       </c>
       <c r="H25" s="1">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I25" s="3">
         <f t="shared" si="2"/>
@@ -1256,7 +1256,7 @@
       </c>
       <c r="J25" s="3">
         <f t="shared" si="2"/>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K25" s="4">
         <v>209</v>

</xml_diff>

<commit_message>
Add line-compare scripts, A35 ENSDF, update stats
Add two comparison utilities (.github/scripts/compare_line_metrics.ps1 and .github/scripts/compare_line_metrics.py) that compute Compare-Object-style line diffs and parse git --numstat output for added/deleted line metrics. Add the A35_revised_2026.ens ENSDF data file (new dataset). Update Statistics.xlsx to reflect related changes. These tools provide both PowerShell and Python implementations to cross-check line-count metrics when comparing files.
</commit_message>
<xml_diff>
--- a/Statistics.xlsx
+++ b/Statistics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\X\ND\ENSDF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A781ADA-B8CF-4AF6-A8A3-CEB3DE3A9724}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B102C3CD-85AC-4444-96FD-81138F1E6112}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{E3F13E08-64ED-4767-9D40-D1E60D65A10A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" activeTab="1" xr2:uid="{E3F13E08-64ED-4767-9D40-D1E60D65A10A}"/>
   </bookViews>
   <sheets>
     <sheet name="A34" sheetId="5" r:id="rId1"/>
@@ -1991,14 +1991,14 @@
         <v>12</v>
       </c>
       <c r="G18" s="1">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="H18" s="1">
         <v>3</v>
       </c>
       <c r="I18" s="3">
         <f t="shared" si="3"/>
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="J18" s="3">
         <f t="shared" si="3"/>
@@ -2032,14 +2032,14 @@
         <v>29</v>
       </c>
       <c r="G19" s="1">
-        <v>379</v>
+        <v>390</v>
       </c>
       <c r="H19" s="1">
         <v>5</v>
       </c>
       <c r="I19" s="3">
         <f t="shared" si="3"/>
-        <v>379</v>
+        <v>390</v>
       </c>
       <c r="J19" s="3">
         <f t="shared" si="3"/>
@@ -2073,14 +2073,14 @@
         <v>34</v>
       </c>
       <c r="G20" s="1">
-        <v>565</v>
+        <v>574</v>
       </c>
       <c r="H20" s="1">
         <v>6</v>
       </c>
       <c r="I20" s="3">
         <f t="shared" si="3"/>
-        <v>565</v>
+        <v>574</v>
       </c>
       <c r="J20" s="3">
         <f t="shared" si="3"/>
@@ -2114,18 +2114,18 @@
         <v>106</v>
       </c>
       <c r="G21" s="1">
-        <v>934</v>
+        <v>925</v>
       </c>
       <c r="H21" s="1">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I21" s="3">
         <f t="shared" si="3"/>
-        <v>934</v>
+        <v>925</v>
       </c>
       <c r="J21" s="3">
         <f t="shared" si="3"/>
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="K21" s="4">
         <v>72</v>
@@ -2155,14 +2155,14 @@
         <v>408</v>
       </c>
       <c r="G22" s="1">
-        <v>2437</v>
+        <v>2456</v>
       </c>
       <c r="H22" s="1">
         <v>14</v>
       </c>
       <c r="I22" s="3">
         <f t="shared" si="3"/>
-        <v>2437</v>
+        <v>2456</v>
       </c>
       <c r="J22" s="3">
         <f t="shared" si="3"/>
@@ -2196,14 +2196,14 @@
         <v>2318</v>
       </c>
       <c r="G23" s="1">
-        <v>8616</v>
+        <v>8930</v>
       </c>
       <c r="H23" s="1">
         <v>28</v>
       </c>
       <c r="I23" s="3">
         <f t="shared" si="3"/>
-        <v>8616</v>
+        <v>8930</v>
       </c>
       <c r="J23" s="3">
         <f t="shared" si="3"/>
@@ -2237,14 +2237,14 @@
         <v>92</v>
       </c>
       <c r="G24" s="1">
-        <v>1232</v>
+        <v>1236</v>
       </c>
       <c r="H24" s="1">
         <v>11</v>
       </c>
       <c r="I24" s="3">
         <f t="shared" si="3"/>
-        <v>1232</v>
+        <v>1236</v>
       </c>
       <c r="J24" s="3">
         <f t="shared" si="3"/>
@@ -2278,14 +2278,14 @@
         <v>0</v>
       </c>
       <c r="G25" s="1">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="H25" s="1">
         <v>3</v>
       </c>
       <c r="I25" s="3">
         <f t="shared" si="3"/>
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J25" s="3">
         <f t="shared" si="3"/>
@@ -2319,14 +2319,14 @@
         <v>0</v>
       </c>
       <c r="G26" s="1">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H26" s="1">
         <v>3</v>
       </c>
       <c r="I26" s="3">
         <f>G26</f>
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="J26" s="3">
         <f>H26</f>
@@ -2360,10 +2360,10 @@
         <v>3003</v>
       </c>
       <c r="G27" s="1">
-        <v>15081</v>
+        <v>15430</v>
       </c>
       <c r="H27" s="1">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I27" s="4"/>
       <c r="J27" s="4"/>

</xml_diff>

<commit_message>
Replace compare_line_metrics.ps1 with Python script
Remove the PowerShell implementation and add a cross-platform Python replacement (.github/scripts/compare_line_metrics.py) that computes Compare-Object-style metrics and git --numstat metrics for two files. The new script:
- Calls PowerShell Compare-Object via subprocess when available, falling back to a Counter-based comparison if needed.
- Invokes git diff --no-index --numstat to obtain added/deleted line counts and reports status/exit code.
- Prints a compact tab-separated summary (OldFile, NewFile, PowerShellTotal/Removed/Added, PowerShellMethod, GitAdded/GitDeleted, GitStatus, GitExitCode).
Default example file paths are included in the script (placeholders). Also updates Statistics.xlsx (binary changed).
</commit_message>
<xml_diff>
--- a/Statistics.xlsx
+++ b/Statistics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\X\ND\ENSDF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B102C3CD-85AC-4444-96FD-81138F1E6112}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EE0A6C8-CFAD-4A09-A853-3823A80ECA39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" activeTab="1" xr2:uid="{E3F13E08-64ED-4767-9D40-D1E60D65A10A}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="73">
   <si>
     <t>Nuclide</t>
   </si>
@@ -189,6 +189,75 @@
   </si>
   <si>
     <t>27NDS</t>
+  </si>
+  <si>
+    <t>OldFile</t>
+  </si>
+  <si>
+    <t>NewFile</t>
+  </si>
+  <si>
+    <t>PowerShellTotal</t>
+  </si>
+  <si>
+    <t>PowerShellRemoved</t>
+  </si>
+  <si>
+    <t>PowerShellAdded</t>
+  </si>
+  <si>
+    <t>PowerShellMethod</t>
+  </si>
+  <si>
+    <t>Compare-Object</t>
+  </si>
+  <si>
+    <t>GitAdded</t>
+  </si>
+  <si>
+    <t>GitDeleted</t>
+  </si>
+  <si>
+    <t>GitStatus</t>
+  </si>
+  <si>
+    <t>ok</t>
+  </si>
+  <si>
+    <t>Nprior</t>
+  </si>
+  <si>
+    <t>ΔNnucl</t>
+  </si>
+  <si>
+    <t>ΔLtotal</t>
+  </si>
+  <si>
+    <t>ΔDset</t>
+  </si>
+  <si>
+    <t>ΔNlevels</t>
+  </si>
+  <si>
+    <t>ΔNgammas</t>
+  </si>
+  <si>
+    <t>NXUNDL</t>
+  </si>
+  <si>
+    <t>Score</t>
+  </si>
+  <si>
+    <t>W</t>
+  </si>
+  <si>
+    <t>A35_NDS2011.txt</t>
+  </si>
+  <si>
+    <t>A35_revised_2026.ens</t>
+  </si>
+  <si>
+    <t>Sum Score</t>
   </si>
 </sst>
 </file>
@@ -220,15 +289,21 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCCECFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -236,11 +311,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -257,6 +347,12 @@
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -265,10 +361,10 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFCCECFF"/>
       <color rgb="FFFF5353"/>
       <color rgb="FFCCFFCC"/>
       <color rgb="FFFFFFCC"/>
-      <color rgb="FFCCECFF"/>
     </mruColors>
   </colors>
   <extLst>
@@ -1467,7 +1563,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AAEAA1E-5B6B-4FC7-9FE5-6150E51A1A48}">
-  <dimension ref="B1:M27"/>
+  <dimension ref="B1:R27"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.44140625" style="1" bestFit="1" customWidth="1"/>
@@ -1482,11 +1578,12 @@
     <col min="12" max="12" width="12.77734375" style="1" customWidth="1"/>
     <col min="13" max="13" width="8.88671875" style="1" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="3.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.21875" style="1" customWidth="1"/>
-    <col min="16" max="16384" width="8.88671875" style="1"/>
+    <col min="15" max="15" width="16.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="17.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1517,7 +1614,7 @@
         <v>#of Datasets</v>
       </c>
     </row>
-    <row r="2" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:18" x14ac:dyDescent="0.3">
       <c r="C2" s="1" t="s">
         <v>9</v>
       </c>
@@ -1538,12 +1635,20 @@
         <v>(non-Adopted)</v>
       </c>
     </row>
-    <row r="3" spans="2:13" ht="12" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:18" ht="12" x14ac:dyDescent="0.3">
       <c r="B3" s="2" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="4" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="O3" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="P3" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q3" s="6"/>
+      <c r="R3" s="6"/>
+    </row>
+    <row r="4" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B4" s="1" t="s">
         <v>14</v>
       </c>
@@ -1573,8 +1678,16 @@
         <f>H4</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="O4" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="P4" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q4" s="6"/>
+      <c r="R4" s="6"/>
+    </row>
+    <row r="5" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B5" s="1" t="s">
         <v>15</v>
       </c>
@@ -1604,8 +1717,16 @@
         <f t="shared" ref="J5:J13" si="1">H5</f>
         <v>3</v>
       </c>
-    </row>
-    <row r="6" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="O5" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="P5" s="6">
+        <v>25032</v>
+      </c>
+      <c r="Q5" s="6"/>
+      <c r="R5" s="6"/>
+    </row>
+    <row r="6" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B6" s="1" t="s">
         <v>16</v>
       </c>
@@ -1635,8 +1756,16 @@
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
-    </row>
-    <row r="7" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="O6" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="P6" s="6">
+        <v>10338</v>
+      </c>
+      <c r="Q6" s="6"/>
+      <c r="R6" s="6"/>
+    </row>
+    <row r="7" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B7" s="1" t="s">
         <v>17</v>
       </c>
@@ -1666,8 +1795,16 @@
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-    </row>
-    <row r="8" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="O7" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="P7" s="6">
+        <v>14694</v>
+      </c>
+      <c r="Q7" s="6"/>
+      <c r="R7" s="6"/>
+    </row>
+    <row r="8" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B8" s="1" t="s">
         <v>3</v>
       </c>
@@ -1697,8 +1834,16 @@
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
-    </row>
-    <row r="9" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="O8" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="P8" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q8" s="6"/>
+      <c r="R8" s="6"/>
+    </row>
+    <row r="9" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B9" s="1" t="s">
         <v>4</v>
       </c>
@@ -1728,8 +1873,16 @@
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-    </row>
-    <row r="10" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="O9" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="P9" s="6">
+        <v>14815</v>
+      </c>
+      <c r="Q9" s="6"/>
+      <c r="R9" s="6"/>
+    </row>
+    <row r="10" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B10" s="1" t="s">
         <v>18</v>
       </c>
@@ -1759,8 +1912,16 @@
         <f t="shared" si="1"/>
         <v>24</v>
       </c>
-    </row>
-    <row r="11" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="O10" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="P10" s="6">
+        <v>10459</v>
+      </c>
+      <c r="Q10" s="6"/>
+      <c r="R10" s="6"/>
+    </row>
+    <row r="11" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B11" s="1" t="s">
         <v>19</v>
       </c>
@@ -1790,8 +1951,16 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-    </row>
-    <row r="12" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="O11" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="P11" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q11" s="6"/>
+      <c r="R11" s="6"/>
+    </row>
+    <row r="12" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B12" s="1" t="s">
         <v>2</v>
       </c>
@@ -1821,8 +1990,12 @@
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-    </row>
-    <row r="13" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="O12" s="6"/>
+      <c r="P12" s="6"/>
+      <c r="Q12" s="6"/>
+      <c r="R12" s="6"/>
+    </row>
+    <row r="13" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B13" s="1" t="s">
         <v>20</v>
       </c>
@@ -1852,8 +2025,12 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="O13" s="6"/>
+      <c r="P13" s="6"/>
+      <c r="Q13" s="6"/>
+      <c r="R13" s="6"/>
+    </row>
+    <row r="14" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B14" s="1" t="s">
         <v>34</v>
       </c>
@@ -1877,8 +2054,16 @@
       </c>
       <c r="I14" s="3"/>
       <c r="J14" s="3"/>
-    </row>
-    <row r="15" spans="2:13" ht="12" x14ac:dyDescent="0.3">
+      <c r="O14" s="6"/>
+      <c r="P14" s="6"/>
+      <c r="Q14" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="R14" s="6" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="15" spans="2:18" ht="12" x14ac:dyDescent="0.3">
       <c r="B15" s="2" t="s">
         <v>38</v>
       </c>
@@ -1891,8 +2076,22 @@
       <c r="M15" s="1" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="16" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="O15" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="P15" s="6">
+        <f>G14</f>
+        <v>11068</v>
+      </c>
+      <c r="Q15" s="6">
+        <v>1E-3</v>
+      </c>
+      <c r="R15" s="6">
+        <f>P15*Q15</f>
+        <v>11.068</v>
+      </c>
+    </row>
+    <row r="16" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B16" s="1" t="s">
         <v>35</v>
       </c>
@@ -1932,8 +2131,21 @@
       <c r="M16" s="4">
         <v>20250509</v>
       </c>
-    </row>
-    <row r="17" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="O16" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="P16" s="6">
+        <v>11</v>
+      </c>
+      <c r="Q16" s="6">
+        <v>1</v>
+      </c>
+      <c r="R16" s="6">
+        <f t="shared" ref="R16:R21" si="3">P16*Q16</f>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B17" s="1" t="s">
         <v>14</v>
       </c>
@@ -1956,11 +2168,11 @@
         <v>2</v>
       </c>
       <c r="I17" s="3">
-        <f t="shared" ref="I17:J25" si="3">G17</f>
+        <f t="shared" ref="I17:J25" si="4">G17</f>
         <v>117</v>
       </c>
       <c r="J17" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="K17" s="4">
@@ -1973,8 +2185,22 @@
       <c r="M17" s="4">
         <v>20250516</v>
       </c>
-    </row>
-    <row r="18" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="O17" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="P17" s="6">
+        <f>P9</f>
+        <v>14815</v>
+      </c>
+      <c r="Q17" s="6">
+        <v>0.02</v>
+      </c>
+      <c r="R17" s="6">
+        <f t="shared" si="3"/>
+        <v>296.3</v>
+      </c>
+    </row>
+    <row r="18" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B18" s="1" t="s">
         <v>15</v>
       </c>
@@ -1997,11 +2223,11 @@
         <v>3</v>
       </c>
       <c r="I18" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>329</v>
       </c>
       <c r="J18" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>3</v>
       </c>
       <c r="K18" s="4">
@@ -2014,8 +2240,22 @@
       <c r="M18" s="4">
         <v>20250528</v>
       </c>
-    </row>
-    <row r="19" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="O18" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="P18" s="6">
+        <f>H27-H14</f>
+        <v>23</v>
+      </c>
+      <c r="Q18" s="6">
+        <v>1</v>
+      </c>
+      <c r="R18" s="6">
+        <f t="shared" si="3"/>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="19" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B19" s="1" t="s">
         <v>16</v>
       </c>
@@ -2038,11 +2278,11 @@
         <v>5</v>
       </c>
       <c r="I19" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>390</v>
       </c>
       <c r="J19" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="K19" s="4">
@@ -2055,8 +2295,22 @@
       <c r="M19" s="4">
         <v>20250603</v>
       </c>
-    </row>
-    <row r="20" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="O19" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="P19" s="6">
+        <f>C27-C14</f>
+        <v>52</v>
+      </c>
+      <c r="Q19" s="6">
+        <v>0.1</v>
+      </c>
+      <c r="R19" s="6">
+        <f t="shared" si="3"/>
+        <v>5.2</v>
+      </c>
+    </row>
+    <row r="20" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B20" s="1" t="s">
         <v>17</v>
       </c>
@@ -2079,11 +2333,11 @@
         <v>6</v>
       </c>
       <c r="I20" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>574</v>
       </c>
       <c r="J20" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>6</v>
       </c>
       <c r="K20" s="4">
@@ -2096,8 +2350,22 @@
       <c r="M20" s="4">
         <v>20250616</v>
       </c>
-    </row>
-    <row r="21" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="O20" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="P20" s="6">
+        <f>D27-D14</f>
+        <v>-52</v>
+      </c>
+      <c r="Q20" s="6">
+        <v>0.1</v>
+      </c>
+      <c r="R20" s="6">
+        <f t="shared" si="3"/>
+        <v>-5.2</v>
+      </c>
+    </row>
+    <row r="21" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B21" s="1" t="s">
         <v>3</v>
       </c>
@@ -2120,11 +2388,11 @@
         <v>11</v>
       </c>
       <c r="I21" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>925</v>
       </c>
       <c r="J21" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>11</v>
       </c>
       <c r="K21" s="4">
@@ -2137,8 +2405,21 @@
       <c r="M21" s="4">
         <v>20250324</v>
       </c>
-    </row>
-    <row r="22" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="O21" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="P21" s="6">
+        <v>42</v>
+      </c>
+      <c r="Q21" s="6">
+        <v>1</v>
+      </c>
+      <c r="R21" s="6">
+        <f t="shared" si="3"/>
+        <v>42</v>
+      </c>
+    </row>
+    <row r="22" spans="2:18" ht="12" x14ac:dyDescent="0.3">
       <c r="B22" s="1" t="s">
         <v>4</v>
       </c>
@@ -2161,11 +2442,11 @@
         <v>14</v>
       </c>
       <c r="I22" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>2456</v>
       </c>
       <c r="J22" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>14</v>
       </c>
       <c r="K22" s="4">
@@ -2178,8 +2459,17 @@
       <c r="M22" s="4">
         <v>20250820</v>
       </c>
-    </row>
-    <row r="23" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="O22" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="P22" s="6"/>
+      <c r="Q22" s="6"/>
+      <c r="R22" s="7">
+        <f>SUM(R15:R21)</f>
+        <v>383.36799999999999</v>
+      </c>
+    </row>
+    <row r="23" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B23" s="1" t="s">
         <v>18</v>
       </c>
@@ -2202,11 +2492,11 @@
         <v>28</v>
       </c>
       <c r="I23" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>8930</v>
       </c>
       <c r="J23" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>28</v>
       </c>
       <c r="K23" s="4">
@@ -2220,7 +2510,7 @@
         <v>20251024</v>
       </c>
     </row>
-    <row r="24" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B24" s="1" t="s">
         <v>19</v>
       </c>
@@ -2243,11 +2533,11 @@
         <v>11</v>
       </c>
       <c r="I24" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1236</v>
       </c>
       <c r="J24" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>11</v>
       </c>
       <c r="K24" s="4">
@@ -2261,7 +2551,7 @@
         <v>20250425</v>
       </c>
     </row>
-    <row r="25" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B25" s="1" t="s">
         <v>2</v>
       </c>
@@ -2284,11 +2574,11 @@
         <v>3</v>
       </c>
       <c r="I25" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>306</v>
       </c>
       <c r="J25" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>3</v>
       </c>
       <c r="K25" s="4">
@@ -2302,7 +2592,7 @@
         <v>20250506</v>
       </c>
     </row>
-    <row r="26" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B26" s="1" t="s">
         <v>20</v>
       </c>
@@ -2343,7 +2633,7 @@
         <v>20250502</v>
       </c>
     </row>
-    <row r="27" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B27" s="1" t="s">
         <v>34</v>
       </c>

</xml_diff>

<commit_message>
Add Cambria font support for Markdown PDF generation; update related scripts and styles
</commit_message>
<xml_diff>
--- a/Statistics.xlsx
+++ b/Statistics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\X\ND\ENSDF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EE0A6C8-CFAD-4A09-A853-3823A80ECA39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4186A527-4BF8-4E9B-8082-D72E4081E0BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" activeTab="1" xr2:uid="{E3F13E08-64ED-4767-9D40-D1E60D65A10A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{E3F13E08-64ED-4767-9D40-D1E60D65A10A}"/>
   </bookViews>
   <sheets>
     <sheet name="A34" sheetId="5" r:id="rId1"/>
@@ -2439,7 +2439,7 @@
         <v>2456</v>
       </c>
       <c r="H22" s="1">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I22" s="3">
         <f t="shared" si="4"/>
@@ -2447,7 +2447,7 @@
       </c>
       <c r="J22" s="3">
         <f t="shared" si="4"/>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K22" s="4">
         <v>309</v>

</xml_diff>